<commit_message>
Default the match key to Item # + Part #
The description is kept as an output column but no longer compared by
default, since wording and capitalisation differ between lists. The
--key option and the workbook dropdown still offer the other keys.
Sample workbooks, expected test rows and README updated to match.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UwZyTGhVQ71zeEDuR3JEHG
</commit_message>
<xml_diff>
--- a/sample_parts.xlsx
+++ b/sample_parts.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Comparison" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Comparison'!$A$1:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Comparison'!$A$1:$G$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -994,7 +994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1005,7 +1005,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="J2" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="J4" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="J6" s="1" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1311,6 +1311,16 @@
           <t>Match</t>
         </is>
       </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Matched on</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Item # + Part #</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1499,69 +1509,38 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>112</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>PN-013</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Pump A</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="5" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Only in List 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>112</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>PN-013</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Pump B</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Only in List 2</t>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Match</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G16"/>
+  <autoFilter ref="A1:G15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>